<commit_message>
Update POSB dashboard and performance reports
</commit_message>
<xml_diff>
--- a/Gudivada_Net_Accounts_Latest.xlsx
+++ b/Gudivada_Net_Accounts_Latest.xlsx
@@ -1022,10 +1022,10 @@
         <v>119</v>
       </c>
       <c r="C14" s="8" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D14" s="9" t="n">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
@@ -1039,10 +1039,10 @@
         <v>125</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>83.2</v>
+        <v>85.59999999999999</v>
       </c>
       <c r="I14" s="11" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="15">
@@ -1807,17 +1807,17 @@
     <row r="38">
       <c r="A38" s="16" t="inlineStr">
         <is>
-          <t>Komaravolu B.O</t>
+          <t>Ponukumada B.O</t>
         </is>
       </c>
       <c r="B38" s="17" t="n">
-        <v>138</v>
+        <v>84</v>
       </c>
       <c r="C38" s="17" t="n">
-        <v>85</v>
+        <v>29</v>
       </c>
       <c r="D38" s="18" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E38" s="16" t="inlineStr">
         <is>
@@ -1831,26 +1831,26 @@
         <v>125</v>
       </c>
       <c r="H38" s="19" t="n">
-        <v>42.4</v>
+        <v>44</v>
       </c>
       <c r="I38" s="11" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="16" t="inlineStr">
         <is>
-          <t>Pedaparupudi B.O</t>
+          <t>Siddantham B.O</t>
         </is>
       </c>
       <c r="B39" s="17" t="n">
-        <v>73</v>
+        <v>132</v>
       </c>
       <c r="C39" s="17" t="n">
-        <v>20</v>
+        <v>78</v>
       </c>
       <c r="D39" s="18" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E39" s="16" t="inlineStr">
         <is>
@@ -1864,23 +1864,23 @@
         <v>125</v>
       </c>
       <c r="H39" s="19" t="n">
-        <v>42.4</v>
+        <v>43.2</v>
       </c>
       <c r="I39" s="11" t="n">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="16" t="inlineStr">
         <is>
-          <t>Ponukumada B.O</t>
+          <t>Komaravolu B.O</t>
         </is>
       </c>
       <c r="B40" s="17" t="n">
-        <v>84</v>
+        <v>138</v>
       </c>
       <c r="C40" s="17" t="n">
-        <v>31</v>
+        <v>85</v>
       </c>
       <c r="D40" s="18" t="n">
         <v>53</v>
@@ -1906,14 +1906,14 @@
     <row r="41">
       <c r="A41" s="16" t="inlineStr">
         <is>
-          <t>Siddantham B.O</t>
+          <t>Pedaparupudi B.O</t>
         </is>
       </c>
       <c r="B41" s="17" t="n">
-        <v>132</v>
+        <v>73</v>
       </c>
       <c r="C41" s="17" t="n">
-        <v>79</v>
+        <v>20</v>
       </c>
       <c r="D41" s="18" t="n">
         <v>53</v>
@@ -2368,14 +2368,14 @@
     <row r="55">
       <c r="A55" s="16" t="inlineStr">
         <is>
-          <t>Serigolvepalli B.O</t>
+          <t>Polukonda B.O</t>
         </is>
       </c>
       <c r="B55" s="17" t="n">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="C55" s="17" t="n">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="D55" s="18" t="n">
         <v>39</v>
@@ -2401,17 +2401,17 @@
     <row r="56">
       <c r="A56" s="16" t="inlineStr">
         <is>
-          <t>Polukonda B.O</t>
+          <t>Serigolvepalli B.O</t>
         </is>
       </c>
       <c r="B56" s="17" t="n">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="C56" s="17" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D56" s="18" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E56" s="16" t="inlineStr">
         <is>
@@ -2425,10 +2425,10 @@
         <v>125</v>
       </c>
       <c r="H56" s="19" t="n">
-        <v>30.4</v>
+        <v>31.2</v>
       </c>
       <c r="I56" s="11" t="n">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="57">
@@ -2870,10 +2870,10 @@
         <v>12</v>
       </c>
       <c r="C70" s="17" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D70" s="18" t="n">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="E70" s="16" t="inlineStr">
         <is>
@@ -2887,10 +2887,10 @@
         <v>125</v>
       </c>
       <c r="H70" s="19" t="n">
-        <v>-1.6</v>
+        <v>-0.8</v>
       </c>
       <c r="I70" s="11" t="n">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="71">
@@ -2993,36 +2993,36 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="16" t="inlineStr">
+      <c r="A74" s="12" t="inlineStr">
         <is>
           <t>Gudivada H.O</t>
         </is>
       </c>
-      <c r="B74" s="17" t="n">
-        <v>1190</v>
-      </c>
-      <c r="C74" s="17" t="n">
-        <v>786</v>
-      </c>
-      <c r="D74" s="18" t="n">
-        <v>404</v>
-      </c>
-      <c r="E74" s="16" t="inlineStr">
+      <c r="B74" s="13" t="n">
+        <v>1191</v>
+      </c>
+      <c r="C74" s="13" t="n">
+        <v>771</v>
+      </c>
+      <c r="D74" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="E74" s="12" t="inlineStr">
         <is>
           <t>HO</t>
         </is>
       </c>
-      <c r="F74" s="17" t="n">
+      <c r="F74" s="13" t="n">
         <v>2000</v>
       </c>
-      <c r="G74" s="17" t="n">
+      <c r="G74" s="13" t="n">
         <v>833.3333333333334</v>
       </c>
-      <c r="H74" s="19" t="n">
-        <v>48.48</v>
+      <c r="H74" s="15" t="n">
+        <v>50.4</v>
       </c>
       <c r="I74" s="11" t="n">
-        <v>429.3333333333334</v>
+        <v>413.3333333333334</v>
       </c>
     </row>
     <row r="75">
@@ -3035,10 +3035,10 @@
         <v>430</v>
       </c>
       <c r="C75" s="3" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D75" s="4" t="n">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
@@ -3052,7 +3052,7 @@
         <v>250</v>
       </c>
       <c r="H75" s="5" t="n">
-        <v>148.8</v>
+        <v>149.2</v>
       </c>
       <c r="I75" s="6" t="n">
         <v>0</v>
@@ -3134,10 +3134,10 @@
         <v>301</v>
       </c>
       <c r="C78" s="3" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D78" s="4" t="n">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
@@ -3151,7 +3151,7 @@
         <v>250</v>
       </c>
       <c r="H78" s="5" t="n">
-        <v>106.4</v>
+        <v>106.8</v>
       </c>
       <c r="I78" s="6" t="n">
         <v>0</v>
@@ -3200,10 +3200,10 @@
         <v>285</v>
       </c>
       <c r="C80" s="8" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D80" s="9" t="n">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="E80" s="7" t="inlineStr">
         <is>
@@ -3217,10 +3217,10 @@
         <v>250</v>
       </c>
       <c r="H80" s="10" t="n">
-        <v>94.8</v>
+        <v>95.19999999999999</v>
       </c>
       <c r="I80" s="11" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="81">
@@ -3233,10 +3233,10 @@
         <v>451</v>
       </c>
       <c r="C81" s="8" t="n">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="D81" s="9" t="n">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="E81" s="7" t="inlineStr">
         <is>
@@ -3250,10 +3250,10 @@
         <v>250</v>
       </c>
       <c r="H81" s="10" t="n">
-        <v>83.59999999999999</v>
+        <v>84.8</v>
       </c>
       <c r="I81" s="11" t="n">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="82">
@@ -3332,10 +3332,10 @@
         <v>341</v>
       </c>
       <c r="C84" s="13" t="n">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="D84" s="14" t="n">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="E84" s="12" t="inlineStr">
         <is>
@@ -3349,10 +3349,10 @@
         <v>250</v>
       </c>
       <c r="H84" s="15" t="n">
-        <v>57.99999999999999</v>
+        <v>58.8</v>
       </c>
       <c r="I84" s="11" t="n">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="85">
@@ -3398,10 +3398,10 @@
         <v>166</v>
       </c>
       <c r="C86" s="17" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D86" s="18" t="n">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E86" s="16" t="inlineStr">
         <is>
@@ -3415,10 +3415,10 @@
         <v>250</v>
       </c>
       <c r="H86" s="19" t="n">
-        <v>46</v>
+        <v>45.6</v>
       </c>
       <c r="I86" s="11" t="n">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="87">
@@ -4000,10 +4000,10 @@
         <v>119</v>
       </c>
       <c r="C14" s="8" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D14" s="9" t="n">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
@@ -4017,10 +4017,10 @@
         <v>125</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>83.2</v>
+        <v>85.59999999999999</v>
       </c>
       <c r="I14" s="11" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="15">
@@ -4785,17 +4785,17 @@
     <row r="38">
       <c r="A38" s="16" t="inlineStr">
         <is>
-          <t>Pedaparupudi B.O</t>
+          <t>Ponukumada B.O</t>
         </is>
       </c>
       <c r="B38" s="17" t="n">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="C38" s="17" t="n">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="D38" s="18" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E38" s="16" t="inlineStr">
         <is>
@@ -4809,26 +4809,26 @@
         <v>125</v>
       </c>
       <c r="H38" s="19" t="n">
-        <v>42.4</v>
+        <v>44</v>
       </c>
       <c r="I38" s="11" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="16" t="inlineStr">
         <is>
-          <t>Veldipadu B.O</t>
+          <t>Siddantham B.O</t>
         </is>
       </c>
       <c r="B39" s="17" t="n">
-        <v>89</v>
+        <v>132</v>
       </c>
       <c r="C39" s="17" t="n">
-        <v>36</v>
+        <v>78</v>
       </c>
       <c r="D39" s="18" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E39" s="16" t="inlineStr">
         <is>
@@ -4842,23 +4842,23 @@
         <v>125</v>
       </c>
       <c r="H39" s="19" t="n">
-        <v>42.4</v>
+        <v>43.2</v>
       </c>
       <c r="I39" s="11" t="n">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="16" t="inlineStr">
         <is>
-          <t>Siddantham B.O</t>
+          <t>Veldipadu B.O</t>
         </is>
       </c>
       <c r="B40" s="17" t="n">
-        <v>132</v>
+        <v>89</v>
       </c>
       <c r="C40" s="17" t="n">
-        <v>79</v>
+        <v>36</v>
       </c>
       <c r="D40" s="18" t="n">
         <v>53</v>
@@ -4884,14 +4884,14 @@
     <row r="41">
       <c r="A41" s="16" t="inlineStr">
         <is>
-          <t>Ponukumada B.O</t>
+          <t>Pedaparupudi B.O</t>
         </is>
       </c>
       <c r="B41" s="17" t="n">
-        <v>84</v>
+        <v>73</v>
       </c>
       <c r="C41" s="17" t="n">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="D41" s="18" t="n">
         <v>53</v>
@@ -5346,14 +5346,14 @@
     <row r="55">
       <c r="A55" s="16" t="inlineStr">
         <is>
-          <t>Serigolvepalli B.O</t>
+          <t>Polukonda B.O</t>
         </is>
       </c>
       <c r="B55" s="17" t="n">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="C55" s="17" t="n">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="D55" s="18" t="n">
         <v>39</v>
@@ -5379,17 +5379,17 @@
     <row r="56">
       <c r="A56" s="16" t="inlineStr">
         <is>
-          <t>Polukonda B.O</t>
+          <t>Serigolvepalli B.O</t>
         </is>
       </c>
       <c r="B56" s="17" t="n">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="C56" s="17" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D56" s="18" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E56" s="16" t="inlineStr">
         <is>
@@ -5403,10 +5403,10 @@
         <v>125</v>
       </c>
       <c r="H56" s="19" t="n">
-        <v>30.4</v>
+        <v>31.2</v>
       </c>
       <c r="I56" s="11" t="n">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="57">
@@ -5848,10 +5848,10 @@
         <v>12</v>
       </c>
       <c r="C70" s="17" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D70" s="18" t="n">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="E70" s="16" t="inlineStr">
         <is>
@@ -5865,10 +5865,10 @@
         <v>125</v>
       </c>
       <c r="H70" s="19" t="n">
-        <v>-1.6</v>
+        <v>-0.8</v>
       </c>
       <c r="I70" s="11" t="n">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="71">
@@ -6054,10 +6054,10 @@
         <v>430</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
@@ -6071,7 +6071,7 @@
         <v>250</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>148.8</v>
+        <v>149.2</v>
       </c>
       <c r="I2" s="6" t="n">
         <v>0</v>
@@ -6153,10 +6153,10 @@
         <v>301</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
@@ -6170,7 +6170,7 @@
         <v>250</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>106.4</v>
+        <v>106.8</v>
       </c>
       <c r="I5" s="6" t="n">
         <v>0</v>
@@ -6219,10 +6219,10 @@
         <v>285</v>
       </c>
       <c r="C7" s="8" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D7" s="9" t="n">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
@@ -6236,10 +6236,10 @@
         <v>250</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>94.8</v>
+        <v>95.19999999999999</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8">
@@ -6252,10 +6252,10 @@
         <v>451</v>
       </c>
       <c r="C8" s="8" t="n">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="D8" s="9" t="n">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
@@ -6269,10 +6269,10 @@
         <v>250</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>83.59999999999999</v>
+        <v>84.8</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="9">
@@ -6351,10 +6351,10 @@
         <v>341</v>
       </c>
       <c r="C11" s="13" t="n">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="E11" s="12" t="inlineStr">
         <is>
@@ -6368,10 +6368,10 @@
         <v>250</v>
       </c>
       <c r="H11" s="15" t="n">
-        <v>57.99999999999999</v>
+        <v>58.8</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="12">
@@ -6417,10 +6417,10 @@
         <v>166</v>
       </c>
       <c r="C13" s="17" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D13" s="18" t="n">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E13" s="16" t="inlineStr">
         <is>
@@ -6434,10 +6434,10 @@
         <v>250</v>
       </c>
       <c r="H13" s="19" t="n">
-        <v>46</v>
+        <v>45.6</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="14">
@@ -6614,36 +6614,36 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="16" t="inlineStr">
+      <c r="A2" s="12" t="inlineStr">
         <is>
           <t>Gudivada H.O</t>
         </is>
       </c>
-      <c r="B2" s="17" t="n">
-        <v>1190</v>
-      </c>
-      <c r="C2" s="17" t="n">
-        <v>786</v>
-      </c>
-      <c r="D2" s="18" t="n">
-        <v>404</v>
-      </c>
-      <c r="E2" s="16" t="inlineStr">
+      <c r="B2" s="13" t="n">
+        <v>1191</v>
+      </c>
+      <c r="C2" s="13" t="n">
+        <v>771</v>
+      </c>
+      <c r="D2" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="E2" s="12" t="inlineStr">
         <is>
           <t>HO</t>
         </is>
       </c>
-      <c r="F2" s="17" t="n">
+      <c r="F2" s="13" t="n">
         <v>2000</v>
       </c>
-      <c r="G2" s="17" t="n">
+      <c r="G2" s="13" t="n">
         <v>833.3333333333334</v>
       </c>
-      <c r="H2" s="19" t="n">
-        <v>48.48</v>
+      <c r="H2" s="15" t="n">
+        <v>50.4</v>
       </c>
       <c r="I2" s="11" t="n">
-        <v>429.3333333333334</v>
+        <v>413.3333333333334</v>
       </c>
     </row>
   </sheetData>
@@ -7068,10 +7068,10 @@
         <v>12</v>
       </c>
       <c r="C5" s="17" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D5" s="18" t="n">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="E5" s="16" t="inlineStr">
         <is>
@@ -7085,10 +7085,10 @@
         <v>125</v>
       </c>
       <c r="H5" s="19" t="n">
-        <v>-1.6</v>
+        <v>-0.8</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="6">
@@ -7208,10 +7208,10 @@
         <v>430</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
@@ -7225,7 +7225,7 @@
         <v>250</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>148.8</v>
+        <v>149.2</v>
       </c>
       <c r="I2" s="6" t="n">
         <v>0</v>
@@ -7517,7 +7517,7 @@
       </c>
       <c r="B2" s="20" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -7568,7 +7568,7 @@
         </is>
       </c>
       <c r="B7" s="21" t="n">
-        <v>12802</v>
+        <v>12803</v>
       </c>
     </row>
     <row r="8">
@@ -7578,7 +7578,7 @@
         </is>
       </c>
       <c r="B8" s="21" t="n">
-        <v>4889</v>
+        <v>4859</v>
       </c>
     </row>
     <row r="9">
@@ -7588,7 +7588,7 @@
         </is>
       </c>
       <c r="B9" s="21" t="n">
-        <v>7913</v>
+        <v>7944</v>
       </c>
     </row>
   </sheetData>

</xml_diff>